<commit_message>
feature: HSCODE 6자리 -> 10자리 구분 및 fallback 로직 추가
</commit_message>
<xml_diff>
--- a/input_template.xlsx
+++ b/input_template.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Sheet1'!$A$1:$I$4</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Sheet1'!$A$1:$J$4</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -470,7 +470,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I4"/>
+  <dimension ref="A1:J4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -479,9 +479,10 @@
     <col width="34" customWidth="1" min="4" max="4"/>
     <col width="24" customWidth="1" min="5" max="5"/>
     <col width="22" customWidth="1" min="6" max="6"/>
-    <col width="34" customWidth="1" min="7" max="7"/>
-    <col width="28" customWidth="1" min="8" max="8"/>
-    <col width="34" customWidth="1" min="9" max="9"/>
+    <col width="22" customWidth="1" min="7" max="7"/>
+    <col width="34" customWidth="1" min="8" max="8"/>
+    <col width="28" customWidth="1" min="9" max="9"/>
+    <col width="34" customWidth="1" min="10" max="10"/>
   </cols>
   <sheetData>
     <row r="1" ht="42" customHeight="1">
@@ -510,22 +511,27 @@
           <t>해당 품목 수출 경험(필수: O/X)</t>
         </is>
       </c>
-      <c r="F1" s="3" t="inlineStr">
-        <is>
-          <t>HS CODE(필수: 6자리 숫자)</t>
+      <c r="F1" s="2" t="inlineStr">
+        <is>
+          <t>HSCODE 10단위(모르는 경우 생략 가능)</t>
         </is>
       </c>
       <c r="G1" s="2" t="inlineStr">
         <is>
+          <t>HSCODE 6단위</t>
+        </is>
+      </c>
+      <c r="H1" s="2" t="inlineStr">
+        <is>
           <t>수출품명(선택: 구체적으로 작성 권장)</t>
         </is>
       </c>
-      <c r="H1" s="2" t="inlineStr">
+      <c r="I1" s="2" t="inlineStr">
         <is>
           <t>희망진출국가(직접분석: 최대 2개, 없으면 공란 가능)</t>
         </is>
       </c>
-      <c r="I1" s="2" t="inlineStr">
+      <c r="J1" s="2" t="inlineStr">
         <is>
           <t>분석 제외 국가(추천보고서: 없으면 공란 가능)</t>
         </is>
@@ -555,22 +561,27 @@
           <t>X</t>
         </is>
       </c>
-      <c r="F2" s="6" t="inlineStr">
+      <c r="F2" s="4" t="inlineStr">
+        <is>
+          <t>3304990000</t>
+        </is>
+      </c>
+      <c r="G2" s="4" t="inlineStr">
         <is>
           <t>330499</t>
         </is>
       </c>
-      <c r="G2" s="5" t="inlineStr">
+      <c r="H2" s="5" t="inlineStr">
         <is>
           <t>스킨케어</t>
         </is>
       </c>
-      <c r="H2" s="4" t="inlineStr">
+      <c r="I2" s="4" t="inlineStr">
         <is>
           <t>베트남, 미국</t>
         </is>
       </c>
-      <c r="I2" s="4" t="inlineStr">
+      <c r="J2" s="4" t="inlineStr">
         <is>
           <t>중국</t>
         </is>
@@ -600,22 +611,23 @@
           <t>O</t>
         </is>
       </c>
-      <c r="F3" s="6" t="inlineStr">
+      <c r="F3" s="4" t="inlineStr"/>
+      <c r="G3" s="4" t="inlineStr">
         <is>
           <t>220600</t>
         </is>
       </c>
-      <c r="G3" s="5" t="inlineStr">
+      <c r="H3" s="5" t="inlineStr">
         <is>
           <t>전통 쌀 발효주(막걸리)</t>
         </is>
       </c>
-      <c r="H3" s="4" t="inlineStr">
+      <c r="I3" s="4" t="inlineStr">
         <is>
           <t>일본</t>
         </is>
       </c>
-      <c r="I3" s="4" t="inlineStr"/>
+      <c r="J3" s="4" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" s="4" t="n">
@@ -641,25 +653,30 @@
           <t>O</t>
         </is>
       </c>
-      <c r="F4" s="6" t="inlineStr">
+      <c r="F4" s="4" t="inlineStr">
+        <is>
+          <t>2103909000</t>
+        </is>
+      </c>
+      <c r="G4" s="4" t="inlineStr">
         <is>
           <t>210390</t>
         </is>
       </c>
-      <c r="G4" s="5" t="inlineStr">
+      <c r="H4" s="5" t="inlineStr">
         <is>
           <t>할랄 비건 콜라겐, 유산균 핫소스</t>
         </is>
       </c>
-      <c r="H4" s="4" t="inlineStr"/>
-      <c r="I4" s="4" t="inlineStr">
+      <c r="I4" s="4" t="inlineStr"/>
+      <c r="J4" s="4" t="inlineStr">
         <is>
           <t>이스라엘</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:I4"/>
+  <autoFilter ref="A1:J4"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>